<commit_message>
School of Leaders 2
</commit_message>
<xml_diff>
--- a/SOL2_DATABASE.xlsx
+++ b/SOL2_DATABASE.xlsx
@@ -20,6 +20,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_CREDITS" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QR_SCANS" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SYSTEM_SETTINGS" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTIFICATIONS" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUEST_VIDEOS" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STUDENT_VIDEO_SUBMISSIONS" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -508,7 +511,11 @@
           <t>Registration Date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="n"/>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>PIN</t>
+        </is>
+      </c>
       <c r="M1" s="1" t="n"/>
       <c r="N1" s="1" t="n"/>
       <c r="O1" s="1" t="n"/>
@@ -848,6 +855,203 @@
       </c>
       <c r="B3" t="n">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Notification ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Table No</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Level No</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Quest No</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Created At</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Read By</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Read At</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Level No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Quest No</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Video Title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Video URL</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Module 1 Prep Video</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Paste a YouTube link here to embed it in the app</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Submission ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Table No</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Level No</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Quest No</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Video URL</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>File Name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>File Size KB</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Submitted At</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>